<commit_message>
Publish the street address: 720 Olive Drive, Suite G, Davis, CA 95616
</commit_message>
<xml_diff>
--- a/openchemworks-sample-sheet.xlsx
+++ b/openchemworks-sample-sheet.xlsx
@@ -569,10 +569,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Amino acid analysis · info@openchemworks.com · Davis, California</t>
-        </is>
-      </c>
-    </row>
+          <t>Amino acid analysis · info@openchemworks.com · 720 Olive Drive, Suite G, Davis, CA 95616</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -580,6 +581,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>

</xml_diff>